<commit_message>
Update data Excel via aplikasi Streamlit
</commit_message>
<xml_diff>
--- a/data_cover.xlsx
+++ b/data_cover.xlsx
@@ -494,10 +494,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -514,10 +512,8 @@
           <t>2016 – 2021</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E2" t="n">
+        <v>10</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -551,10 +547,8 @@
       <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -571,10 +565,8 @@
           <t>2022-ON</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E3" t="n">
+        <v>10</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -608,10 +600,8 @@
       <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -628,10 +618,8 @@
           <t>2021-ON</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
+      <c r="E4" t="n">
+        <v>3</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -665,10 +653,8 @@
       <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -685,10 +671,8 @@
           <t>2006-2013</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
+      <c r="E5" t="n">
+        <v>5</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -722,10 +706,8 @@
       <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -742,10 +724,8 @@
           <t>2014-2017</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
+      <c r="E6" t="n">
+        <v>4</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -779,10 +759,8 @@
       <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="A7" t="n">
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -799,10 +777,8 @@
           <t>2023-ON</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
+      <c r="E7" t="n">
+        <v>9</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -836,10 +812,8 @@
       <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="A8" t="n">
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -856,10 +830,8 @@
           <t xml:space="preserve">2017 – 2020 </t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>08</t>
-        </is>
+      <c r="E8" t="n">
+        <v>8</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -893,10 +865,8 @@
       <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="A9" t="n">
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -913,10 +883,8 @@
           <t>2021 – 2023</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>08</t>
-        </is>
+      <c r="E9" t="n">
+        <v>8</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -950,10 +918,8 @@
       <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+      <c r="A10" t="n">
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -970,10 +936,8 @@
           <t>1998-2007</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="E10" t="n">
+        <v>14</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1007,10 +971,8 @@
       <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="A11" t="n">
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1027,10 +989,8 @@
           <t>2019-2024</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="E11" t="n">
+        <v>13</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1064,10 +1024,8 @@
       <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="A12" t="n">
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1084,10 +1042,8 @@
           <t>2012-2018</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
+      <c r="E12" t="n">
+        <v>6</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1121,10 +1077,8 @@
       <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="A13" t="n">
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1141,10 +1095,8 @@
           <t>2022-ON</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E13" t="n">
+        <v>10</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1178,10 +1130,8 @@
       <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="A14" t="n">
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1198,10 +1148,8 @@
           <t>2022-ON</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E14" t="n">
+        <v>10</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1231,10 +1179,8 @@
       <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="A15" t="n">
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1251,10 +1197,8 @@
           <t>2001 – 2007</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
+      <c r="E15" t="n">
+        <v>6</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1288,10 +1232,8 @@
       <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="A16" t="n">
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1308,10 +1250,8 @@
           <t>2008 – 2013</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
+      <c r="E16" t="n">
+        <v>6</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1345,10 +1285,8 @@
       <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="A17" t="n">
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1365,10 +1303,8 @@
           <t>2014 – 2019</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
+      <c r="E17" t="n">
+        <v>6</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1402,10 +1338,8 @@
       <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
+      <c r="A18" t="n">
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1422,10 +1356,8 @@
           <t>2019-ON</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
+      <c r="E18" t="n">
+        <v>6</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1459,10 +1391,8 @@
       <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="A19" t="n">
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1479,10 +1409,8 @@
           <t>1950 – 1967</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="E19" t="n">
+        <v>16</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1516,10 +1444,8 @@
       <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
+      <c r="A20" t="n">
+        <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1536,10 +1462,8 @@
           <t>1967 – 1979</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="E20" t="n">
+        <v>16</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1573,10 +1497,8 @@
       <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="A21" t="n">
+        <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1593,10 +1515,8 @@
           <t>2002–2014</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="E21" t="n">
+        <v>14</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1630,10 +1550,8 @@
       <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
+      <c r="A22" t="n">
+        <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1650,10 +1568,8 @@
           <t>2015-ON</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="E22" t="n">
+        <v>14</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1687,10 +1603,8 @@
       <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+      <c r="A23" t="n">
+        <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1707,10 +1621,8 @@
           <t>2007-2021</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="E23" t="n">
+        <v>11</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1744,10 +1656,8 @@
       <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="A24" t="n">
+        <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1764,10 +1674,8 @@
           <t>2022-ON</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="E24" t="n">
+        <v>14</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1801,10 +1709,8 @@
       <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="A25" t="n">
+        <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1821,10 +1727,8 @@
           <t>2018-ON</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="E25" t="n">
+        <v>13</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1862,10 +1766,8 @@
       <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
+      <c r="A26" t="n">
+        <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1882,10 +1784,8 @@
           <t>2014–2018</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="E26" t="n">
+        <v>13</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1923,10 +1823,8 @@
       <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+      <c r="A27" t="n">
+        <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1943,10 +1841,8 @@
           <t>2013–2022</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
+      <c r="E27" t="n">
+        <v>2</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1980,10 +1876,8 @@
       <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
+      <c r="A28" t="n">
+        <v>27</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2000,10 +1894,8 @@
           <t>2023–ON</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
+      <c r="E28" t="n">
+        <v>2</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -2053,10 +1945,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="A29" t="n">
+        <v>28</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2073,10 +1963,8 @@
           <t>1974–1980</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
+      <c r="E29" t="n">
+        <v>3</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -2114,10 +2002,8 @@
       <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="A30" t="n">
+        <v>29</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2134,10 +2020,8 @@
           <t>1981–1992</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
+      <c r="E30" t="n">
+        <v>4</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -2179,10 +2063,8 @@
       <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="A31" t="n">
+        <v>30</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2199,10 +2081,8 @@
           <t>1984 ke atas</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
+      <c r="E31" t="n">
+        <v>4</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -2240,10 +2120,8 @@
       <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="A32" t="n">
+        <v>31</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2260,10 +2138,8 @@
           <t>2008–2017</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
+      <c r="E32" t="n">
+        <v>4</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -2305,10 +2181,8 @@
       <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
+      <c r="A33" t="n">
+        <v>32</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2325,10 +2199,8 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E33" t="n">
+        <v>10</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -2366,10 +2238,8 @@
       <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="A34" t="n">
+        <v>33</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2386,10 +2256,8 @@
           <t>2004 – 2019</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
+      <c r="E34" t="n">
+        <v>5</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2431,10 +2299,8 @@
       <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
+      <c r="A35" t="n">
+        <v>34</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2451,10 +2317,8 @@
           <t xml:space="preserve">2004 – 2012 </t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
+      <c r="E35" t="n">
+        <v>4</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2496,10 +2360,8 @@
       <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="A36" t="n">
+        <v>35</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2516,10 +2378,8 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="E36" t="n">
+        <v>13</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2561,10 +2421,8 @@
       <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
+      <c r="A37" t="n">
+        <v>36</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2581,10 +2439,8 @@
           <t>2022-2026</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
+      <c r="E37" t="n">
+        <v>9</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2626,10 +2482,8 @@
       <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="A38" t="n">
+        <v>37</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2646,10 +2500,8 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
+      <c r="E38" t="n">
+        <v>3</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2691,10 +2543,8 @@
       <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
+      <c r="A39" t="n">
+        <v>38</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2711,10 +2561,8 @@
           <t>2023</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="E39" t="n">
+        <v>14</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2756,10 +2604,8 @@
       <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="A40" t="n">
+        <v>39</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2776,10 +2622,8 @@
           <t>2017–2020</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E40" t="n">
+        <v>10</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2821,10 +2665,8 @@
       <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="A41" t="n">
+        <v>40</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -2841,10 +2683,8 @@
           <t>2021–2026</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E41" t="n">
+        <v>10</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2886,10 +2726,8 @@
       <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
+      <c r="A42" t="n">
+        <v>41</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2906,10 +2744,8 @@
           <t>2019-On</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
+      <c r="E42" t="n">
+        <v>9</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2955,10 +2791,8 @@
       <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
+      <c r="A43" t="n">
+        <v>42</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2975,10 +2809,8 @@
           <t>2022-On</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E43" t="n">
+        <v>10</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -3024,10 +2856,8 @@
       <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
+      <c r="A44" t="n">
+        <v>43</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3044,10 +2874,8 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="E44" t="n">
+        <v>13</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -3089,10 +2917,8 @@
       <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
+      <c r="A45" t="n">
+        <v>44</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3109,10 +2935,8 @@
           <t xml:space="preserve">2025 (2024 Cina) </t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
+      <c r="E45" t="n">
+        <v>17</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>

</xml_diff>